<commit_message>
feat: Phase 9 - M1 Core Operations
</commit_message>
<xml_diff>
--- a/QS-WFUI-Info.xlsx
+++ b/QS-WFUI-Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\00 CIPAA contract work dairy\QS-WFUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26318067-13C2-4FA1-99C5-D443DD6BBF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D45FA5-7C24-4BA0-877D-CEBE37A72366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t>MyQSWFUI16071995#</t>
   </si>
@@ -350,6 +350,72 @@
   </si>
   <si>
     <t>After Sprint 10 you'll have a complete, demo-ready BOQ-to-RFQ workflow — Stage 1 of the roadmap done for real. That's the right moment for the first public demo.</t>
+  </si>
+  <si>
+    <t>pnpm dev in apps/api)</t>
+  </si>
+  <si>
+    <r>
+      <t>contractor-admin@lados.dev</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → admin</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>contractor-driver1@lados.dev</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → driver</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>contractor-driver2@lados.dev</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → driver</t>
+    </r>
+  </si>
+  <si>
+    <t>4 auth users with pre-confirmed email/password</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> contractor-owner@lados.dev → owner</t>
+  </si>
+  <si>
+    <t>eeeeeeee-0001-0000-0000-000000000001</t>
+  </si>
+  <si>
+    <t>Syarikat Bina Jaya Sdn Bhd</t>
+  </si>
+  <si>
+    <t>c09f14c5-59e0-4be2-b0a8-d62691695a6f</t>
+  </si>
+  <si>
+    <t>test123</t>
   </si>
 </sst>
 </file>
@@ -416,7 +482,6 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -430,6 +495,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -710,11 +776,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E11"/>
+  <dimension ref="A2:E27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="48.85546875" customWidth="1"/>
     <col min="4" max="4" width="38.42578125" customWidth="1"/>
   </cols>
@@ -723,7 +789,7 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
@@ -777,11 +843,56 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" s="4"/>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5">
+      <c r="B26" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5">
+      <c r="B27" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -798,7 +909,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:2" ht="18">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>16</v>
       </c>
     </row>
@@ -808,109 +919,109 @@
       </c>
     </row>
     <row r="6" spans="2:2">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" spans="2:2">
-      <c r="B7" s="5"/>
+      <c r="B7" s="4"/>
     </row>
     <row r="8" spans="2:2">
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="2:2">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="2:2">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11" spans="2:2">
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="2:2">
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="14" spans="2:2">
-      <c r="B14" s="5"/>
+      <c r="B14" s="4"/>
     </row>
     <row r="15" spans="2:2">
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" spans="2:2">
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="17" spans="2:2">
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="19" spans="2:2">
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="20" spans="2:2">
-      <c r="B20" s="5"/>
+      <c r="B20" s="4"/>
     </row>
     <row r="21" spans="2:2">
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="5" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="22" spans="2:2">
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="23" spans="2:2">
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="24" spans="2:2">
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="26" spans="2:2">
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="27" spans="2:2">
-      <c r="B27" s="5"/>
+      <c r="B27" s="4"/>
     </row>
     <row r="28" spans="2:2">
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="29" spans="2:2">
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="4" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="30" spans="2:2">
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="4" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="31" spans="2:2">
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="4" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: icon/emoji display + naming consistency across packs
</commit_message>
<xml_diff>
--- a/QS-WFUI-Info.xlsx
+++ b/QS-WFUI-Info.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\00 CIPAA contract work dairy\QS-WFUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F61B4E57-EFD4-4087-9803-262780524EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D83A2B15-744C-4CF2-AF51-60F0DCFA2AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="105">
   <si>
     <t>MyQSWFUI16071995#</t>
   </si>
@@ -352,9 +353,6 @@
     <t>After Sprint 10 you'll have a complete, demo-ready BOQ-to-RFQ workflow — Stage 1 of the roadmap done for real. That's the right moment for the first public demo.</t>
   </si>
   <si>
-    <t>pnpm dev in apps/api)</t>
-  </si>
-  <si>
     <r>
       <t>contractor-admin@lados.dev</t>
     </r>
@@ -428,13 +426,610 @@
   </si>
   <si>
     <t xml:space="preserve"> https://console.upstash.com/redis</t>
+  </si>
+  <si>
+    <t>pnpm dev in apps/api</t>
+  </si>
+  <si>
+    <t>pnpm dev in apps/web</t>
+  </si>
+  <si>
+    <t>localhost 3000</t>
+  </si>
+  <si>
+    <t>localhost 4000</t>
+  </si>
+  <si>
+    <t>⚠️ PARTIALLY TRUE / OVERSTATED</t>
+  </si>
+  <si>
+    <t>"Manifest-driven Inspector"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PropertyPanel.tsx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (653 lines) is NOT fully manifest-driven. Phase 4A added </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ResourcePickerField</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and some manifest-awareness, but the panel is largely hardcoded per field type. A true manifest-driven inspector would read a node's manifest </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>parameters</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> array and auto-render the correct field components. What exists is a good start, not the spec claim.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Typed connections" on canvas</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Node manifests declare </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ports.inputs[].type</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ports.outputs[].type</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, but </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>WorkflowCanvas.tsx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> does NOT enforce type compatibility during drag connections. There is no </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>isValidConnection</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> callback checking port types. Users can connect any output to any input. The typed ports exist in metadata only.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Explorer + Canvas + Inspector" separation</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The document describes three separate panels (Explorer / Canvas / Inspector). What exists: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>NodePalette</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (sidebar node browser), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>WorkflowCanvas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (canvas), and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>PropertyPanel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (inspector). There is no component named </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Explorer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and the NodePalette is much simpler than what a full Explorer implies (no resource browser, no template browser, no execution browser). Canvas and Inspector are real.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Node search"</t>
+  </si>
+  <si>
+    <r>
+      <t>NodePalette</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> has category filtering and text filtering — but no fuzzy search, no keyboard shortcut search-to-add (like ComfyUI's double-click), no tag-based search.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Workflow JSON V2"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The shared type is </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>QSWorkflowDefinition</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (QS from the old @qsos namespace). It functions as V2 in spirit but is not explicitly versioned as such in the type name. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>@lados/workflow-json</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> package exists with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>validateWorkflow()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>WorkflowBuilder</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Frontend State Engine"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The document mentions "LCE State Engine plus frontend state engine." The backend State Engine is real. The frontend has no dedicated state engine — it uses standard React </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>useState</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>useEffect</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. No XState, no Zustand, no Redux. This is aspirational.</t>
+    </r>
+  </si>
+  <si>
+    <t>❌ NOT YET IMPLEMENTED / ASPIRATIONAL</t>
+  </si>
+  <si>
+    <t>Resource Bindings</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The document states </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Workspace Resource → Workflow Binding → Node Reference</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. There is no </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>resource_bindings</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table in any migration. Workflow nodes do not formally bind to workspace resources through a binding layer. Resources exist as standalone domain objects, but nodes don't reference them via a governed binding mechanism. The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ResourcePickerField</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in PropertyPanel stores a resource ID in node config directly — not a proper binding. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>This is the biggest gap between the documents and reality.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Marketplace distribution" externally</t>
+  </si>
+  <si>
+    <t>The pack marketplace is a local install system (enable/disable compiled packs). There is no external registry, no pack upload, no public distribution. The document's "Native Pack Marketplace" claim is accurate only for the local install story.</t>
+  </si>
+  <si>
+    <t>"Generated from Manifest UI Schema"</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The ComfyUI comparison specifically claims "Generated from Manifest UI Schema" vs ComfyUI's "Hardcoded node UI." This is not true yet. PropertyPanel renders fields based on hardcoded logic, not dynamically generated from each node's manifest </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>parameters</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> array.</t>
+    </r>
+  </si>
+  <si>
+    <t>"Multi-tenant Support" (full isolation)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Org-level access control works via </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>organization_members</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> roles, but row-level security (RLS) policies in Supabase are not consistently applied across all tables — the API uses the service role admin client everywhere, bypassing RLS. True multi-tenant isolation at the DB level is partial.</t>
+    </r>
+  </si>
+  <si>
+    <t>Summary Table</t>
+  </si>
+  <si>
+    <t>Document Claim</t>
+  </si>
+  <si>
+    <t>Reality</t>
+  </si>
+  <si>
+    <t>Workspace → Project → Workflow model</t>
+  </si>
+  <si>
+    <t>✅ True</t>
+  </si>
+  <si>
+    <t>Node Manifest V2 + executor</t>
+  </si>
+  <si>
+    <t>Pack SDK</t>
+  </si>
+  <si>
+    <t>Execution versioning</t>
+  </si>
+  <si>
+    <t>Native approvals + pause/resume</t>
+  </si>
+  <si>
+    <t>✅ True (stronger than claimed)</t>
+  </si>
+  <si>
+    <t>Live execution feedback</t>
+  </si>
+  <si>
+    <t>✅ True (SSE, not polling)</t>
+  </si>
+  <si>
+    <t>Event Bus</t>
+  </si>
+  <si>
+    <t>Audit Trail</t>
+  </si>
+  <si>
+    <t>Backend State Engine</t>
+  </si>
+  <si>
+    <t>Business Resources</t>
+  </si>
+  <si>
+    <t>Multi-user org-aware</t>
+  </si>
+  <si>
+    <t>Manifest-driven Inspector</t>
+  </si>
+  <si>
+    <t>⚠️ Partial — hardcoded, not auto-generated</t>
+  </si>
+  <si>
+    <t>Typed connection enforcement</t>
+  </si>
+  <si>
+    <t>⚠️ Partial — types in manifests only</t>
+  </si>
+  <si>
+    <t>Explorer (full)</t>
+  </si>
+  <si>
+    <t>⚠️ Partial — NodePalette only</t>
+  </si>
+  <si>
+    <t>Frontend State Engine</t>
+  </si>
+  <si>
+    <t>❌ Not implemented</t>
+  </si>
+  <si>
+    <t>Resource Bindings (formal layer)</t>
+  </si>
+  <si>
+    <t>UI generated from Manifest UI Schema</t>
+  </si>
+  <si>
+    <t>External Marketplace distribution</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -471,6 +1066,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -492,7 +1101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -507,7 +1116,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -864,69 +1482,81 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>54</v>
+      </c>
       <c r="B17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="B22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="B23" s="4"/>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="B24" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E24" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="B25" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="2:5">
-      <c r="B22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" t="s">
+    <row r="26" spans="1:5">
+      <c r="B26" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="B27" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="B30" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D22" t="s">
+      <c r="C30" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="2:5">
-      <c r="B23" s="4"/>
-    </row>
-    <row r="24" spans="2:5">
-      <c r="B24" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" t="s">
-        <v>48</v>
-      </c>
-      <c r="D24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E24" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5">
-      <c r="B25" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5">
-      <c r="B26" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5">
-      <c r="B27" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5">
-      <c r="B30" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C30" t="s">
-        <v>50</v>
-      </c>
-    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1064,4 +1694,285 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9CFEE9D-DAF6-487D-AF39-D1944A98CC9B}">
+  <dimension ref="B3:C61"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="46.140625" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:2" ht="15.75">
+      <c r="B3" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2">
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2">
+      <c r="B8" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2">
+      <c r="B9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2">
+      <c r="B11" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2">
+      <c r="B12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2">
+      <c r="B14" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2">
+      <c r="B15" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" ht="15.75">
+      <c r="B25" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2">
+      <c r="B27" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3">
+      <c r="B33" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3">
+      <c r="B34" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3">
+      <c r="B36" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3">
+      <c r="B37" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" ht="15.75">
+      <c r="B41" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3">
+      <c r="B43" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3">
+      <c r="B44" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3">
+      <c r="B45" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="46" spans="2:3">
+      <c r="B46" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="47" spans="2:3">
+      <c r="B47" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="48" spans="2:3" ht="30">
+      <c r="B48" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3">
+      <c r="B49" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3">
+      <c r="B50" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3">
+      <c r="B51" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3">
+      <c r="B52" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="53" spans="2:3">
+      <c r="B53" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="54" spans="2:3">
+      <c r="B54" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="55" spans="2:3" ht="30">
+      <c r="B55" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="56" spans="2:3" ht="30">
+      <c r="B56" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="2:3" ht="30">
+      <c r="B57" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="58" spans="2:3">
+      <c r="B58" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="59" spans="2:3">
+      <c r="B59" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="60" spans="2:3">
+      <c r="B60" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="61" spans="2:3">
+      <c r="B61" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>